<commit_message>
mejoras indicador compuesto y gráficos
</commit_message>
<xml_diff>
--- a/Resultados_Ajuste_Mercado_Financiero.xlsx
+++ b/Resultados_Ajuste_Mercado_Financiero.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Datos Completos" sheetId="1" state="visible" r:id="rId2"/>
@@ -1046,7 +1046,7 @@
         <v>0.845045917506116</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
         <v>19</v>
       </c>
@@ -1095,7 +1095,7 @@
         <v>0.808910656767043</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
         <v>19</v>
       </c>
@@ -1144,7 +1144,7 @@
         <v>0.92452847219878</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
         <v>19</v>
       </c>
@@ -1193,7 +1193,7 @@
         <v>0.924594361553132</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
         <v>19</v>
       </c>
@@ -1242,7 +1242,7 @@
         <v>0.63881807861339</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
         <v>19</v>
       </c>
@@ -1291,7 +1291,7 @@
         <v>0.845045917506116</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
         <v>19</v>
       </c>
@@ -1340,7 +1340,7 @@
         <v>0.71861778335103</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
         <v>19</v>
       </c>
@@ -1389,7 +1389,7 @@
         <v>0.000587997250029392</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
         <v>20</v>
       </c>
@@ -1438,7 +1438,7 @@
         <v>0.312103917237801</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
         <v>20</v>
       </c>
@@ -1458,7 +1458,7 @@
         <v>0.920382192558499</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>1.82948863293718</v>
+        <v>1.82</v>
       </c>
       <c r="I47" s="2" t="n">
         <v>0.212812646626988</v>
@@ -1487,7 +1487,7 @@
         <v>0.382474064632232</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
         <v>20</v>
       </c>
@@ -1536,7 +1536,7 @@
         <v>0.000338585313287854</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
         <v>20</v>
       </c>
@@ -1585,7 +1585,7 @@
         <v>0.00758501887826366</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
         <v>20</v>
       </c>
@@ -1634,7 +1634,7 @@
         <v>0.000587997250029392</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
         <v>20</v>
       </c>
@@ -1683,7 +1683,7 @@
         <v>0.274968788172407</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
         <v>20</v>
       </c>
@@ -2061,7 +2061,7 @@
     </filterColumn>
     <filterColumn colId="0">
       <customFilters and="true">
-        <customFilter operator="equal" val="19 meses"/>
+        <customFilter operator="equal" val="3 meses"/>
       </customFilters>
     </filterColumn>
   </autoFilter>
@@ -2447,7 +2447,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G36"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -3294,7 +3294,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E36"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -3924,8 +3924,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q33"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:Q34"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.16"/>
   </cols>

</xml_diff>